<commit_message>
mean difference and figure aesthetics
</commit_message>
<xml_diff>
--- a/output/tables/pfratio_12h_by_treatment_obs.xlsx
+++ b/output/tables/pfratio_12h_by_treatment_obs.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t xml:space="preserve">Time Since Randomisation (hours)
 </t>
@@ -22,6 +22,9 @@
   </si>
   <si>
     <t xml:space="preserve">Welch Two Sample t-test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abbreviation: CI = Confidence Interval</t>
   </si>
   <si>
     <t xml:space="preserve">Observations
@@ -102,6 +105,47 @@
   </si>
   <si>
     <t xml:space="preserve">27.06 (9.24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean Difference
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">95% CI
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-7.61, -0.63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.73, -0.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.79, -0.32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.98, 1.36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.81, -0.17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.41, 0.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.65, 2.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.21, 2.64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.87, 3.24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-6.94, 0.38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.29, 0.64</t>
   </si>
   <si>
     <t xml:space="preserve">p-value
@@ -550,6 +594,8 @@
     <col min="3" max="3" width="10.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="10.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="10.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="10.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="10.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="NA" customHeight="1">
@@ -557,16 +603,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="2" ht="NA" customHeight="1">
@@ -577,12 +629,18 @@
         <v>217</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" s="7" t="n">
+        <v>-4.12</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" s="7" t="n">
         <v>0.021</v>
       </c>
     </row>
@@ -594,12 +652,18 @@
         <v>309</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="8" t="n">
+        <v>-2.74</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="8" t="n">
         <v>0.007</v>
       </c>
     </row>
@@ -611,12 +675,18 @@
         <v>295</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" s="8" t="n">
+        <v>-2.55</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="8" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -628,12 +698,18 @@
         <v>245</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" s="8" t="n">
+        <v>-1.81</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="8" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -645,12 +721,18 @@
         <v>257</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E6" s="8" t="n">
+        <v>-2.49</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="8" t="n">
         <v>0.036</v>
       </c>
     </row>
@@ -662,12 +744,18 @@
         <v>244</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E7" s="8" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="8" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -679,12 +767,18 @@
         <v>227</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="8" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" s="8" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -696,12 +790,18 @@
         <v>208</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" s="8" t="n">
+        <v>-0.79</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="8" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -713,13 +813,19 @@
         <v>213</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>29</v>
+        <v>26</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="11" ht="NA" customHeight="1">
@@ -730,12 +836,18 @@
         <v>174</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E11" s="8" t="n">
+        <v>-3.28</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="G11" s="8" t="n">
         <v>0.078</v>
       </c>
     </row>
@@ -747,12 +859,18 @@
         <v>176</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E12" s="9" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="9" t="n">
         <v>0.12</v>
       </c>
     </row>
@@ -772,28 +890,64 @@
       <c r="E13" s="5" t="s">
         <v>1</v>
       </c>
+      <c r="F13" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" ht="NA" customHeight="1">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="4" t="s">
         <v>2</v>
       </c>
+      <c r="F14" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="NA" customHeight="1">
+      <c r="A15" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A14:E14"/>
+  <mergeCells count="3">
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Plymouth data and renv
</commit_message>
<xml_diff>
--- a/output/tables/pfratio_12h_by_treatment_obs.xlsx
+++ b/output/tables/pfratio_12h_by_treatment_obs.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">Time Since Randomisation (hours)
 </t>
@@ -32,79 +32,79 @@
   </si>
   <si>
     <t xml:space="preserve">Conservative
-N = 1,258
+N = 1,356
 </t>
   </si>
   <si>
-    <t xml:space="preserve">22.72 (12.76)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.89 (8.60)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.49 (9.52)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.38 (14.39)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.15 (8.23)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.41 (8.91)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.07 (10.16)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.57 (9.81)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.09 (10.88)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.17 (11.47)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.74 (10.66)</t>
+    <t xml:space="preserve">22.24 (12.40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.67 (8.50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.46 (9.49)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.87 (14.01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.93 (8.59)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.80 (9.01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.45 (10.20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.71 (9.79)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.11 (10.92)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.65 (11.25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.70 (10.60)</t>
   </si>
   <si>
     <t xml:space="preserve">Usual care
-N = 1,307
+N = 1,556
 </t>
   </si>
   <si>
-    <t xml:space="preserve">26.84 (13.32)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.63 (9.14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29.05 (9.95)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29.19 (10.23)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28.64 (10.62)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.41 (10.17)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28.34 (15.04)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.35 (14.78)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.90 (11.70)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.45 (12.82)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.06 (9.24)</t>
+    <t xml:space="preserve">26.13 (13.28)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.09 (9.36)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.99 (9.77)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.56 (10.01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29.40 (15.74)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.77 (10.33)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.75 (14.56)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.21 (14.02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30.00 (24.57)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.16 (12.26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.52 (10.13)</t>
   </si>
   <si>
     <t xml:space="preserve">Mean Difference
@@ -115,44 +115,41 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">-7.61, -0.63</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.73, -0.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.79, -0.32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.98, 1.36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.81, -0.17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.41, 0.40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.65, 2.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.21, 2.64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.87, 3.24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-6.94, 0.38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-5.29, 0.64</t>
+    <t xml:space="preserve">-7.20, -0.57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.29, 0.47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.62, 0.56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.58, 1.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-6.29, -0.66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.24, 0.30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.35, 1.76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.54, 1.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-8.57, 0.79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-6.81, -0.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.89, 0.25</t>
   </si>
   <si>
     <t xml:space="preserve">p-value
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">&gt;0.9</t>
   </si>
 </sst>
 </file>
@@ -626,7 +623,7 @@
         <v>-12</v>
       </c>
       <c r="B2" s="7" t="n">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>6</v>
@@ -635,13 +632,13 @@
         <v>18</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>-4.12</v>
+        <v>-3.89</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>31</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>0.021</v>
+        <v>0.022</v>
       </c>
     </row>
     <row r="3" ht="NA" customHeight="1">
@@ -649,7 +646,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="8" t="n">
-        <v>309</v>
+        <v>350</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>7</v>
@@ -658,13 +655,13 @@
         <v>19</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>-2.74</v>
+        <v>-1.41</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>32</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>0.007</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="4" ht="NA" customHeight="1">
@@ -672,7 +669,7 @@
         <v>12</v>
       </c>
       <c r="B4" s="8" t="n">
-        <v>295</v>
+        <v>333</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>8</v>
@@ -681,13 +678,13 @@
         <v>20</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>-2.55</v>
+        <v>-1.53</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>0.025</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5" ht="NA" customHeight="1">
@@ -695,7 +692,7 @@
         <v>24</v>
       </c>
       <c r="B5" s="8" t="n">
-        <v>245</v>
+        <v>289</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>9</v>
@@ -704,13 +701,13 @@
         <v>21</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>-1.81</v>
+        <v>-1.69</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>34</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6" ht="NA" customHeight="1">
@@ -718,7 +715,7 @@
         <v>36</v>
       </c>
       <c r="B6" s="8" t="n">
-        <v>257</v>
+        <v>301</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>10</v>
@@ -727,13 +724,13 @@
         <v>22</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>-2.49</v>
+        <v>-3.48</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>35</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0.036</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="7" ht="NA" customHeight="1">
@@ -741,7 +738,7 @@
         <v>48</v>
       </c>
       <c r="B7" s="8" t="n">
-        <v>244</v>
+        <v>282</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>11</v>
@@ -750,13 +747,13 @@
         <v>23</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>-2</v>
+        <v>-1.97</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>36</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.1</v>
+        <v>0.089</v>
       </c>
     </row>
     <row r="8" ht="NA" customHeight="1">
@@ -764,7 +761,7 @@
         <v>60</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>227</v>
+        <v>259</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>12</v>
@@ -773,13 +770,13 @@
         <v>24</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>-1.27</v>
+        <v>-1.3</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>37</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="9" ht="NA" customHeight="1">
@@ -787,7 +784,7 @@
         <v>72</v>
       </c>
       <c r="B9" s="8" t="n">
-        <v>208</v>
+        <v>241</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>13</v>
@@ -796,13 +793,13 @@
         <v>25</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>-0.79</v>
+        <v>-1.5</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>38</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="10" ht="NA" customHeight="1">
@@ -810,7 +807,7 @@
         <v>84</v>
       </c>
       <c r="B10" s="8" t="n">
-        <v>213</v>
+        <v>248</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>14</v>
@@ -819,13 +816,13 @@
         <v>26</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>0.19</v>
+        <v>-3.89</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>43</v>
+      <c r="G10" s="8" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="11" ht="NA" customHeight="1">
@@ -833,7 +830,7 @@
         <v>96</v>
       </c>
       <c r="B11" s="8" t="n">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>15</v>
@@ -842,13 +839,13 @@
         <v>27</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>-3.28</v>
+        <v>-3.51</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>0.078</v>
+        <v>0.037</v>
       </c>
     </row>
     <row r="12" ht="NA" customHeight="1">
@@ -856,7 +853,7 @@
         <v>108</v>
       </c>
       <c r="B12" s="9" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>16</v>
@@ -865,13 +862,13 @@
         <v>28</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>-2.32</v>
+        <v>-2.82</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>41</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>0.12</v>
+        <v>0.071</v>
       </c>
     </row>
     <row r="13" ht="NA" customHeight="1">

</xml_diff>

<commit_message>
added P14 and figure parameters
</commit_message>
<xml_diff>
--- a/output/tables/pfratio_12h_by_treatment_obs.xlsx
+++ b/output/tables/pfratio_12h_by_treatment_obs.xlsx
@@ -18,93 +18,18 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Mean (SD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Welch Two Sample t-test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abbreviation: CI = Confidence Interval</t>
-  </si>
-  <si>
     <t xml:space="preserve">Observations
 </t>
   </si>
   <si>
     <t xml:space="preserve">Conservative
-N = 1,356
+N = 1,335
 </t>
   </si>
   <si>
-    <t xml:space="preserve">22.24 (12.40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.67 (8.50)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.46 (9.49)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.87 (14.01)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.93 (8.59)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.80 (9.01)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.45 (10.20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.71 (9.79)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.11 (10.92)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23.65 (11.25)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.70 (10.60)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Usual care
-N = 1,556
+N = 1,589
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.13 (13.28)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.09 (9.36)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.99 (9.77)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28.56 (10.01)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29.40 (15.74)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.77 (10.33)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.75 (14.56)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.21 (14.02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30.00 (24.57)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.16 (12.26)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.52 (10.13)</t>
   </si>
   <si>
     <t xml:space="preserve">Mean Difference
@@ -115,41 +40,116 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">-7.20, -0.57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3.29, 0.47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3.62, 0.56</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.58, 1.20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-6.29, -0.66</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.24, 0.30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.35, 1.76</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.54, 1.54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-8.57, 0.79</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-6.81, -0.21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-5.89, 0.25</t>
-  </si>
-  <si>
     <t xml:space="preserve">p-value
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.29 (11.92)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.46 (13.08)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-8.26, -2.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.36 (8.43)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.52 (9.66)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.07, -0.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.01 (9.40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.43 (9.93)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.53, -0.31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.50 (7.77)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29.11 (11.70)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.88, -1.32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.70 (8.62)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29.57 (15.81)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-6.70, -1.03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.24 (8.71)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.99 (10.41)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.01, -0.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.03 (10.17)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.61 (14.48)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.64, 1.49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.62 (9.79)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.14 (13.80)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.52, 1.48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.11 (10.92)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29.71 (24.24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-8.21, 0.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.65 (11.25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.50 (12.13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-7.10, -0.61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.70 (10.60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.49 (9.28)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.71, 0.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean (SD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welch Two Sample t-test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abbreviation: CI = Confidence Interval</t>
   </si>
 </sst>
 </file>
@@ -600,22 +600,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>30</v>
-      </c>
       <c r="G1" s="6" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" ht="NA" customHeight="1">
@@ -623,22 +623,22 @@
         <v>-12</v>
       </c>
       <c r="B2" s="7" t="n">
-        <v>233</v>
+        <v>255</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>-3.89</v>
+        <v>-5.17</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>0.022</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="3" ht="NA" customHeight="1">
@@ -649,19 +649,19 @@
         <v>350</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>-1.41</v>
+        <v>-2.17</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>0.14</v>
+        <v>0.026</v>
       </c>
     </row>
     <row r="4" ht="NA" customHeight="1">
@@ -669,22 +669,22 @@
         <v>12</v>
       </c>
       <c r="B4" s="8" t="n">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>-1.53</v>
+        <v>-2.42</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>0.2</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="5" ht="NA" customHeight="1">
@@ -692,22 +692,22 @@
         <v>24</v>
       </c>
       <c r="B5" s="8" t="n">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>-1.69</v>
+        <v>-3.6</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>0.2</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="6" ht="NA" customHeight="1">
@@ -715,22 +715,22 @@
         <v>36</v>
       </c>
       <c r="B6" s="8" t="n">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>-3.48</v>
+        <v>-3.87</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0.016</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="7" ht="NA" customHeight="1">
@@ -738,22 +738,22 @@
         <v>48</v>
       </c>
       <c r="B7" s="8" t="n">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>-1.97</v>
+        <v>-2.75</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.089</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="8" ht="NA" customHeight="1">
@@ -761,22 +761,22 @@
         <v>60</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>-1.3</v>
+        <v>-1.57</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="9" ht="NA" customHeight="1">
@@ -784,19 +784,19 @@
         <v>72</v>
       </c>
       <c r="B9" s="8" t="n">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>-1.5</v>
+        <v>-1.52</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>0.3</v>
@@ -807,22 +807,22 @@
         <v>84</v>
       </c>
       <c r="B10" s="8" t="n">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>-3.89</v>
+        <v>-3.61</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="11" ht="NA" customHeight="1">
@@ -830,22 +830,22 @@
         <v>96</v>
       </c>
       <c r="B11" s="8" t="n">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>-3.51</v>
+        <v>-3.86</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>0.037</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="12" ht="NA" customHeight="1">
@@ -853,91 +853,91 @@
         <v>108</v>
       </c>
       <c r="B12" s="9" t="n">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>-2.82</v>
+        <v>-2.79</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>0.071</v>
+        <v>0.061</v>
       </c>
     </row>
     <row r="13" ht="NA" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" ht="NA" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" ht="NA" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>